<commit_message>
Updated dataset after review
</commit_message>
<xml_diff>
--- a/Data/dispersion_and_reaction_data.xlsx
+++ b/Data/dispersion_and_reaction_data.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trarg\Documents\SM\SM Experiment\DATA\Stats\Regression_Model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1505D7D6-2F6C-4612-93F6-5362282B7974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D1C2EF-213E-4AF3-B7D7-75FA29E6834C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D1CF5FF3-BC6E-4FF7-BE4B-16ADEB7A652E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D1CF5FF3-BC6E-4FF7-BE4B-16ADEB7A652E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!#REF!</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$B$109</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Fatigue</t>
   </si>
@@ -88,6 +87,9 @@
   </si>
   <si>
     <t>Reacted_Before_TOR</t>
+  </si>
+  <si>
+    <t>Event_Number</t>
   </si>
 </sst>
 </file>
@@ -439,10 +441,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9F0F03B-9386-4C50-90B6-016F7CF3CBF2}">
-  <dimension ref="A1:P106"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:Q109"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -491,8 +494,11 @@
       <c r="P1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -541,8 +547,11 @@
       <c r="P2">
         <v>5.5230890039716813</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -591,8 +600,11 @@
       <c r="P3">
         <v>8.9323006430941607</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -641,8 +653,11 @@
       <c r="P4">
         <v>1.842987674861047</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1</v>
       </c>
@@ -691,8 +706,11 @@
       <c r="P5">
         <v>7.7312116808799347</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1</v>
       </c>
@@ -741,8 +759,11 @@
       <c r="P6">
         <v>4.3888627840547345</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1</v>
       </c>
@@ -791,8 +812,11 @@
       <c r="P7">
         <v>9.0902131399397099</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
@@ -841,8 +865,11 @@
       <c r="P8">
         <v>8.269028542040898</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1</v>
       </c>
@@ -891,8 +918,11 @@
       <c r="P9">
         <v>5.6257265434475743</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1</v>
       </c>
@@ -941,8 +971,11 @@
       <c r="P10">
         <v>6.4483921799510222</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1</v>
       </c>
@@ -991,8 +1024,11 @@
       <c r="P11">
         <v>6.5250172063448577</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1</v>
       </c>
@@ -1041,8 +1077,11 @@
       <c r="P12">
         <v>7.7265007645925907</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1</v>
       </c>
@@ -1091,8 +1130,11 @@
       <c r="P13">
         <v>3.1520253234246907</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1</v>
       </c>
@@ -1141,8 +1183,11 @@
       <c r="P14">
         <v>6.0944769520396251</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1</v>
       </c>
@@ -1191,8 +1236,11 @@
       <c r="P15">
         <v>5.8428370396860405</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>1</v>
       </c>
@@ -1241,8 +1289,11 @@
       <c r="P16">
         <v>5.3892953946952824</v>
       </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1</v>
       </c>
@@ -1291,8 +1342,11 @@
       <c r="P17">
         <v>1.1459155902616465</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>1</v>
       </c>
@@ -1341,8 +1395,11 @@
       <c r="P18">
         <v>7.2810659567409166</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1</v>
       </c>
@@ -1391,8 +1448,11 @@
       <c r="P19">
         <v>7.9759478528726504</v>
       </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1</v>
       </c>
@@ -1441,8 +1501,11 @@
       <c r="P20">
         <v>8.7656460135062861</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1</v>
       </c>
@@ -1491,8 +1554,11 @@
       <c r="P21">
         <v>6.4200497912908432</v>
       </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>1</v>
       </c>
@@ -1541,8 +1607,11 @@
       <c r="P22">
         <v>8.8698957989218972</v>
       </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>1</v>
       </c>
@@ -1591,8 +1660,11 @@
       <c r="P23">
         <v>7.5455515828613331</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>1</v>
       </c>
@@ -1641,8 +1713,11 @@
       <c r="P24">
         <v>8.3543316444955646</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>1</v>
       </c>
@@ -1691,8 +1766,11 @@
       <c r="P25">
         <v>5.2312669884877776</v>
       </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>1</v>
       </c>
@@ -1741,8 +1819,11 @@
       <c r="P26">
         <v>5.1190319475772057</v>
       </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>1</v>
       </c>
@@ -1791,8 +1872,11 @@
       <c r="P27">
         <v>8.3605617583767007</v>
       </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>1</v>
       </c>
@@ -1841,8 +1925,11 @@
       <c r="P28">
         <v>5.7372366208599654</v>
       </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>1</v>
       </c>
@@ -1891,8 +1978,11 @@
       <c r="P29">
         <v>4.8197962019989857</v>
       </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>1</v>
       </c>
@@ -1941,8 +2031,11 @@
       <c r="P30">
         <v>7.9657045134113007</v>
       </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>1</v>
       </c>
@@ -1991,8 +2084,11 @@
       <c r="P31">
         <v>7.0326451504634946</v>
       </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>1</v>
       </c>
@@ -2041,8 +2137,11 @@
       <c r="P32">
         <v>8.7135228969676426</v>
       </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>1</v>
       </c>
@@ -2091,8 +2190,11 @@
       <c r="P33">
         <v>7.8241221731636728</v>
       </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>1</v>
       </c>
@@ -2141,8 +2243,11 @@
       <c r="P34">
         <v>6.63672134456246</v>
       </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>1</v>
       </c>
@@ -2191,8 +2296,11 @@
       <c r="P35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>1</v>
       </c>
@@ -2241,8 +2349,11 @@
       <c r="P36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>1</v>
       </c>
@@ -2291,8 +2402,11 @@
       <c r="P37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>1</v>
       </c>
@@ -2341,8 +2455,11 @@
       <c r="P38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>1</v>
       </c>
@@ -2391,8 +2508,11 @@
       <c r="P39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>1</v>
       </c>
@@ -2441,8 +2561,11 @@
       <c r="P40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q40">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>1</v>
       </c>
@@ -2491,8 +2614,11 @@
       <c r="P41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q41">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>1</v>
       </c>
@@ -2541,8 +2667,11 @@
       <c r="P42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>1</v>
       </c>
@@ -2591,8 +2720,11 @@
       <c r="P43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>1</v>
       </c>
@@ -2641,8 +2773,11 @@
       <c r="P44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>1</v>
       </c>
@@ -2691,8 +2826,11 @@
       <c r="P45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>1</v>
       </c>
@@ -2741,8 +2879,11 @@
       <c r="P46">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>1</v>
       </c>
@@ -2791,8 +2932,11 @@
       <c r="P47">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q47">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>1</v>
       </c>
@@ -2841,8 +2985,11 @@
       <c r="P48">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q48">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>1</v>
       </c>
@@ -2891,8 +3038,11 @@
       <c r="P49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>1</v>
       </c>
@@ -2941,8 +3091,11 @@
       <c r="P50">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q50">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>1</v>
       </c>
@@ -2991,8 +3144,11 @@
       <c r="P51">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q51">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>1</v>
       </c>
@@ -3041,8 +3197,11 @@
       <c r="P52">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q52">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>1</v>
       </c>
@@ -3091,8 +3250,11 @@
       <c r="P53">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>1</v>
       </c>
@@ -3141,8 +3303,11 @@
       <c r="P54">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>1</v>
       </c>
@@ -3191,8 +3356,11 @@
       <c r="P55">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q55">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>1</v>
       </c>
@@ -3241,8 +3409,11 @@
       <c r="P56">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q56">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>1</v>
       </c>
@@ -3291,8 +3462,11 @@
       <c r="P57">
         <v>0</v>
       </c>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>1</v>
       </c>
@@ -3341,8 +3515,11 @@
       <c r="P58">
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q58">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>1</v>
       </c>
@@ -3391,8 +3568,11 @@
       <c r="P59">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>1</v>
       </c>
@@ -3441,8 +3621,11 @@
       <c r="P60">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>1</v>
       </c>
@@ -3491,8 +3674,11 @@
       <c r="P61">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q61">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>1</v>
       </c>
@@ -3541,8 +3727,11 @@
       <c r="P62">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>1</v>
       </c>
@@ -3591,8 +3780,11 @@
       <c r="P63">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>1</v>
       </c>
@@ -3641,8 +3833,11 @@
       <c r="P64">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q64">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>1</v>
       </c>
@@ -3691,8 +3886,11 @@
       <c r="P65">
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q65">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>1</v>
       </c>
@@ -3741,8 +3939,11 @@
       <c r="P66">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q66">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>1</v>
       </c>
@@ -3791,8 +3992,11 @@
       <c r="P67">
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>1</v>
       </c>
@@ -3841,8 +4045,11 @@
       <c r="P68">
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q68">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>1</v>
       </c>
@@ -3891,8 +4098,11 @@
       <c r="P69">
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q69">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>1</v>
       </c>
@@ -3941,8 +4151,11 @@
       <c r="P70">
         <v>5.4449291955320271</v>
       </c>
-    </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q70">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>1</v>
       </c>
@@ -3991,8 +4204,11 @@
       <c r="P71">
         <v>8.2750666004691027</v>
       </c>
-    </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>1</v>
       </c>
@@ -4041,8 +4257,11 @@
       <c r="P72">
         <v>7.3136842148345957</v>
       </c>
-    </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q72">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>1</v>
       </c>
@@ -4091,8 +4310,11 @@
       <c r="P73">
         <v>7.4221074821257202</v>
       </c>
-    </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q73">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>1</v>
       </c>
@@ -4141,8 +4363,11 @@
       <c r="P74">
         <v>5.5833902335991219</v>
       </c>
-    </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>1</v>
       </c>
@@ -4191,8 +4416,11 @@
       <c r="P75">
         <v>5.0722443286183818</v>
       </c>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q75">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>1</v>
       </c>
@@ -4241,8 +4469,11 @@
       <c r="P76">
         <v>7.6237681141227052</v>
       </c>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>1</v>
       </c>
@@ -4291,8 +4522,11 @@
       <c r="P77">
         <v>6.4198716014165571</v>
       </c>
-    </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q77">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>1</v>
       </c>
@@ -4341,8 +4575,11 @@
       <c r="P78">
         <v>4.6776867978756167</v>
       </c>
-    </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>1</v>
       </c>
@@ -4391,8 +4628,11 @@
       <c r="P79">
         <v>8.6737749239586943</v>
       </c>
-    </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q79">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>1</v>
       </c>
@@ -4441,8 +4681,11 @@
       <c r="P80">
         <v>8.053302541018585</v>
       </c>
-    </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q80">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>1</v>
       </c>
@@ -4491,8 +4734,11 @@
       <c r="P81">
         <v>7.1540173785161354</v>
       </c>
-    </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>1</v>
       </c>
@@ -4541,8 +4787,11 @@
       <c r="P82">
         <v>4.136613760269146</v>
       </c>
-    </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q82">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>1</v>
       </c>
@@ -4591,8 +4840,11 @@
       <c r="P83">
         <v>3.6816445909318189</v>
       </c>
-    </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q83">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>1</v>
       </c>
@@ -4641,8 +4893,11 @@
       <c r="P84">
         <v>5.0576163150382349</v>
       </c>
-    </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q84">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>1</v>
       </c>
@@ -4691,13 +4946,16 @@
       <c r="P85">
         <v>2.9046915326761913</v>
       </c>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q85">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>1</v>
       </c>
       <c r="B86">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C86">
         <v>3</v>
@@ -4709,266 +4967,281 @@
         <v>1</v>
       </c>
       <c r="F86">
-        <v>1.32</v>
+        <v>2.23</v>
       </c>
       <c r="G86">
         <v>0.21</v>
       </c>
       <c r="H86">
-        <v>0.25</v>
+        <v>0.21</v>
       </c>
       <c r="I86">
         <v>12.032113697747288</v>
       </c>
       <c r="J86">
+        <v>12.032113697747288</v>
+      </c>
+      <c r="K86">
+        <v>0</v>
+      </c>
+      <c r="L86">
+        <v>1</v>
+      </c>
+      <c r="M86">
+        <v>0.160054637</v>
+      </c>
+      <c r="N86">
+        <v>0.162121971</v>
+      </c>
+      <c r="O86">
+        <v>9.1704551915984283</v>
+      </c>
+      <c r="P86">
+        <v>9.2889047046423272</v>
+      </c>
+      <c r="Q86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>1</v>
+      </c>
+      <c r="B87">
+        <v>1</v>
+      </c>
+      <c r="C87">
+        <v>3</v>
+      </c>
+      <c r="D87">
+        <v>1</v>
+      </c>
+      <c r="E87">
+        <v>1</v>
+      </c>
+      <c r="F87">
+        <v>1.83</v>
+      </c>
+      <c r="G87">
+        <v>0.11</v>
+      </c>
+      <c r="H87">
+        <v>0.18</v>
+      </c>
+      <c r="I87">
+        <v>6.3025357464390552</v>
+      </c>
+      <c r="J87">
+        <v>10.313240312354818</v>
+      </c>
+      <c r="K87">
+        <v>0</v>
+      </c>
+      <c r="L87">
+        <v>1</v>
+      </c>
+      <c r="M87">
+        <v>0.19846751800000001</v>
+      </c>
+      <c r="N87">
+        <v>0.18295019200000001</v>
+      </c>
+      <c r="O87">
+        <v>11.371351151836697</v>
+      </c>
+      <c r="P87">
+        <v>10.482273862708078</v>
+      </c>
+      <c r="Q87">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>1</v>
+      </c>
+      <c r="B88">
+        <v>1</v>
+      </c>
+      <c r="C88">
+        <v>3</v>
+      </c>
+      <c r="D88">
+        <v>1</v>
+      </c>
+      <c r="E88">
+        <v>1</v>
+      </c>
+      <c r="F88">
+        <v>1.58</v>
+      </c>
+      <c r="G88">
+        <v>0.17</v>
+      </c>
+      <c r="H88">
+        <v>0.22</v>
+      </c>
+      <c r="I88">
+        <v>9.7402825172239957</v>
+      </c>
+      <c r="J88">
+        <v>12.60507149287811</v>
+      </c>
+      <c r="K88">
+        <v>0</v>
+      </c>
+      <c r="L88">
+        <v>0</v>
+      </c>
+      <c r="M88">
+        <v>0.185135622</v>
+      </c>
+      <c r="N88">
+        <v>0.14476037899999999</v>
+      </c>
+      <c r="O88">
+        <v>10.607489778129352</v>
+      </c>
+      <c r="P88">
+        <v>8.2941587574142321</v>
+      </c>
+      <c r="Q88">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>1</v>
+      </c>
+      <c r="B89">
+        <v>0</v>
+      </c>
+      <c r="C89">
+        <v>3</v>
+      </c>
+      <c r="D89">
+        <v>1</v>
+      </c>
+      <c r="E89">
+        <v>1</v>
+      </c>
+      <c r="F89">
+        <v>1.32</v>
+      </c>
+      <c r="G89">
+        <v>0.21</v>
+      </c>
+      <c r="H89">
+        <v>0.25</v>
+      </c>
+      <c r="I89">
+        <v>12.032113697747288</v>
+      </c>
+      <c r="J89">
         <v>14.323944878270581</v>
       </c>
-      <c r="K86">
-        <v>0</v>
-      </c>
-      <c r="L86">
-        <v>0</v>
-      </c>
-      <c r="M86">
+      <c r="K89">
+        <v>0</v>
+      </c>
+      <c r="L89">
+        <v>0</v>
+      </c>
+      <c r="M89">
         <v>6.7867026999999996E-2</v>
       </c>
-      <c r="N86">
+      <c r="N89">
         <v>5.4583408999999999E-2</v>
       </c>
-      <c r="O86">
+      <c r="O89">
         <v>3.8884942152004047</v>
       </c>
-      <c r="P86">
+      <c r="P89">
         <v>3.1273989671363931</v>
       </c>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A87">
-        <v>1</v>
-      </c>
-      <c r="B87">
-        <v>0</v>
-      </c>
-      <c r="C87">
-        <v>3</v>
-      </c>
-      <c r="D87">
-        <v>1</v>
-      </c>
-      <c r="E87">
-        <v>1</v>
-      </c>
-      <c r="F87">
+      <c r="Q89">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>1</v>
+      </c>
+      <c r="B90">
+        <v>0</v>
+      </c>
+      <c r="C90">
+        <v>3</v>
+      </c>
+      <c r="D90">
+        <v>1</v>
+      </c>
+      <c r="E90">
+        <v>1</v>
+      </c>
+      <c r="F90">
         <v>1.64</v>
       </c>
-      <c r="G87">
+      <c r="G90">
         <v>0.22</v>
       </c>
-      <c r="H87">
+      <c r="H90">
         <v>0.28000000000000003</v>
       </c>
-      <c r="I87">
+      <c r="I90">
         <v>12.60507149287811</v>
       </c>
-      <c r="J87">
+      <c r="J90">
         <v>16.042818263663051</v>
       </c>
-      <c r="K87">
-        <v>0</v>
-      </c>
-      <c r="L87">
-        <v>0</v>
-      </c>
-      <c r="M87">
+      <c r="K90">
+        <v>0</v>
+      </c>
+      <c r="L90">
+        <v>0</v>
+      </c>
+      <c r="M90">
         <v>0.16657482300000001</v>
       </c>
-      <c r="N87">
+      <c r="N90">
         <v>0.14517633999999999</v>
       </c>
-      <c r="O87">
+      <c r="O90">
         <v>9.5440343310387146</v>
       </c>
-      <c r="P87">
+      <c r="P90">
         <v>8.3179915671562732</v>
       </c>
-    </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A88">
-        <v>1</v>
-      </c>
-      <c r="B88">
-        <v>0</v>
-      </c>
-      <c r="C88">
-        <v>3</v>
-      </c>
-      <c r="D88">
-        <v>1</v>
-      </c>
-      <c r="E88">
-        <v>1</v>
-      </c>
-      <c r="F88">
+      <c r="Q90">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A91">
+        <v>1</v>
+      </c>
+      <c r="B91">
+        <v>0</v>
+      </c>
+      <c r="C91">
+        <v>3</v>
+      </c>
+      <c r="D91">
+        <v>1</v>
+      </c>
+      <c r="E91">
+        <v>1</v>
+      </c>
+      <c r="F91">
         <v>2.13</v>
       </c>
-      <c r="G88">
+      <c r="G91">
         <v>0.22</v>
-      </c>
-      <c r="H88">
-        <v>0.21</v>
-      </c>
-      <c r="I88">
-        <v>12.60507149287811</v>
-      </c>
-      <c r="J88">
-        <v>12.032113697747288</v>
-      </c>
-      <c r="K88">
-        <v>0</v>
-      </c>
-      <c r="L88">
-        <v>0</v>
-      </c>
-      <c r="M88">
-        <v>0.108891636</v>
-      </c>
-      <c r="N88">
-        <v>0.102433514</v>
-      </c>
-      <c r="O88">
-        <v>6.2390311670748169</v>
-      </c>
-      <c r="P88">
-        <v>5.8690080328942313</v>
-      </c>
-    </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A89">
-        <v>1</v>
-      </c>
-      <c r="B89">
-        <v>0</v>
-      </c>
-      <c r="C89">
-        <v>3</v>
-      </c>
-      <c r="D89">
-        <v>1</v>
-      </c>
-      <c r="E89">
-        <v>1</v>
-      </c>
-      <c r="F89">
-        <v>2.75</v>
-      </c>
-      <c r="G89">
-        <v>0.2</v>
-      </c>
-      <c r="H89">
-        <v>0.23</v>
-      </c>
-      <c r="I89">
-        <v>11.459155902616466</v>
-      </c>
-      <c r="J89">
-        <v>13.178029288008934</v>
-      </c>
-      <c r="K89">
-        <v>0</v>
-      </c>
-      <c r="L89">
-        <v>1</v>
-      </c>
-      <c r="M89">
-        <v>0.12278276</v>
-      </c>
-      <c r="N89">
-        <v>0.16339498599999999</v>
-      </c>
-      <c r="O89">
-        <v>7.0349339449677037</v>
-      </c>
-      <c r="P89">
-        <v>9.361843091399173</v>
-      </c>
-    </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A90">
-        <v>1</v>
-      </c>
-      <c r="B90">
-        <v>0</v>
-      </c>
-      <c r="C90">
-        <v>3</v>
-      </c>
-      <c r="D90">
-        <v>1</v>
-      </c>
-      <c r="E90">
-        <v>1</v>
-      </c>
-      <c r="F90">
-        <v>2.16</v>
-      </c>
-      <c r="G90">
-        <v>0.15</v>
-      </c>
-      <c r="H90">
-        <v>0.17</v>
-      </c>
-      <c r="I90">
-        <v>8.5943669269623477</v>
-      </c>
-      <c r="J90">
-        <v>9.7402825172239957</v>
-      </c>
-      <c r="K90">
-        <v>0</v>
-      </c>
-      <c r="L90">
-        <v>1</v>
-      </c>
-      <c r="M90">
-        <v>0.19412848299999999</v>
-      </c>
-      <c r="N90">
-        <v>0.15817606000000001</v>
-      </c>
-      <c r="O90">
-        <v>11.12274275917715</v>
-      </c>
-      <c r="P90">
-        <v>9.0628206580080803</v>
-      </c>
-    </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A91">
-        <v>1</v>
-      </c>
-      <c r="B91">
-        <v>0</v>
-      </c>
-      <c r="C91">
-        <v>3</v>
-      </c>
-      <c r="D91">
-        <v>1</v>
-      </c>
-      <c r="E91">
-        <v>1</v>
-      </c>
-      <c r="F91">
-        <v>2.35</v>
-      </c>
-      <c r="G91">
-        <v>0.17</v>
       </c>
       <c r="H91">
         <v>0.21</v>
       </c>
       <c r="I91">
-        <v>9.7402825172239957</v>
+        <v>12.60507149287811</v>
       </c>
       <c r="J91">
         <v>12.032113697747288</v>
@@ -4980,495 +5253,525 @@
         <v>0</v>
       </c>
       <c r="M91">
+        <v>0.108891636</v>
+      </c>
+      <c r="N91">
+        <v>0.102433514</v>
+      </c>
+      <c r="O91">
+        <v>6.2390311670748169</v>
+      </c>
+      <c r="P91">
+        <v>5.8690080328942313</v>
+      </c>
+      <c r="Q91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>1</v>
+      </c>
+      <c r="B92">
+        <v>0</v>
+      </c>
+      <c r="C92">
+        <v>3</v>
+      </c>
+      <c r="D92">
+        <v>1</v>
+      </c>
+      <c r="E92">
+        <v>1</v>
+      </c>
+      <c r="F92">
+        <v>2.75</v>
+      </c>
+      <c r="G92">
+        <v>0.2</v>
+      </c>
+      <c r="H92">
+        <v>0.23</v>
+      </c>
+      <c r="I92">
+        <v>11.459155902616466</v>
+      </c>
+      <c r="J92">
+        <v>13.178029288008934</v>
+      </c>
+      <c r="K92">
+        <v>0</v>
+      </c>
+      <c r="L92">
+        <v>1</v>
+      </c>
+      <c r="M92">
+        <v>0.12278276</v>
+      </c>
+      <c r="N92">
+        <v>0.16339498599999999</v>
+      </c>
+      <c r="O92">
+        <v>7.0349339449677037</v>
+      </c>
+      <c r="P92">
+        <v>9.361843091399173</v>
+      </c>
+      <c r="Q92">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>1</v>
+      </c>
+      <c r="B93">
+        <v>0</v>
+      </c>
+      <c r="C93">
+        <v>3</v>
+      </c>
+      <c r="D93">
+        <v>1</v>
+      </c>
+      <c r="E93">
+        <v>1</v>
+      </c>
+      <c r="F93">
+        <v>2.16</v>
+      </c>
+      <c r="G93">
+        <v>0.15</v>
+      </c>
+      <c r="H93">
+        <v>0.17</v>
+      </c>
+      <c r="I93">
+        <v>8.5943669269623477</v>
+      </c>
+      <c r="J93">
+        <v>9.7402825172239957</v>
+      </c>
+      <c r="K93">
+        <v>0</v>
+      </c>
+      <c r="L93">
+        <v>1</v>
+      </c>
+      <c r="M93">
+        <v>0.19412848299999999</v>
+      </c>
+      <c r="N93">
+        <v>0.15817606000000001</v>
+      </c>
+      <c r="O93">
+        <v>11.12274275917715</v>
+      </c>
+      <c r="P93">
+        <v>9.0628206580080803</v>
+      </c>
+      <c r="Q93">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>1</v>
+      </c>
+      <c r="B94">
+        <v>0</v>
+      </c>
+      <c r="C94">
+        <v>3</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
+      </c>
+      <c r="E94">
+        <v>1</v>
+      </c>
+      <c r="F94">
+        <v>2.35</v>
+      </c>
+      <c r="G94">
+        <v>0.17</v>
+      </c>
+      <c r="H94">
+        <v>0.21</v>
+      </c>
+      <c r="I94">
+        <v>9.7402825172239957</v>
+      </c>
+      <c r="J94">
+        <v>12.032113697747288</v>
+      </c>
+      <c r="K94">
+        <v>0</v>
+      </c>
+      <c r="L94">
+        <v>0</v>
+      </c>
+      <c r="M94">
         <v>0.180473462</v>
       </c>
-      <c r="N91">
+      <c r="N94">
         <v>0.15584858400000001</v>
       </c>
-      <c r="O91">
+      <c r="O94">
         <v>10.340367686714639</v>
       </c>
-      <c r="P91">
+      <c r="P94">
         <v>8.9294661062900893</v>
       </c>
-    </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A92">
-        <v>1</v>
-      </c>
-      <c r="B92">
-        <v>0</v>
-      </c>
-      <c r="C92">
-        <v>3</v>
-      </c>
-      <c r="D92">
-        <v>1</v>
-      </c>
-      <c r="E92">
-        <v>1</v>
-      </c>
-      <c r="F92">
+      <c r="Q94">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A95">
+        <v>1</v>
+      </c>
+      <c r="B95">
+        <v>0</v>
+      </c>
+      <c r="C95">
+        <v>3</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95">
+        <v>1</v>
+      </c>
+      <c r="F95">
         <v>1.98</v>
       </c>
-      <c r="G92">
+      <c r="G95">
         <v>0.18</v>
       </c>
-      <c r="H92">
+      <c r="H95">
         <v>0.18</v>
       </c>
-      <c r="I92">
+      <c r="I95">
         <v>10.313240312354818</v>
       </c>
-      <c r="J92">
+      <c r="J95">
         <v>10.313240312354818</v>
       </c>
-      <c r="K92">
-        <v>0</v>
-      </c>
-      <c r="L92">
-        <v>0</v>
-      </c>
-      <c r="M92">
+      <c r="K95">
+        <v>0</v>
+      </c>
+      <c r="L95">
+        <v>0</v>
+      </c>
+      <c r="M95">
         <v>0.203938018</v>
       </c>
-      <c r="N92">
+      <c r="N95">
         <v>0.14337982099999999</v>
       </c>
-      <c r="O92">
+      <c r="O95">
         <v>11.684787713663015</v>
       </c>
-      <c r="P92">
+      <c r="P95">
         <v>8.2150586106412096</v>
       </c>
-    </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A93">
-        <v>1</v>
-      </c>
-      <c r="B93">
-        <v>0</v>
-      </c>
-      <c r="C93">
-        <v>3</v>
-      </c>
-      <c r="D93">
-        <v>1</v>
-      </c>
-      <c r="E93">
-        <v>1</v>
-      </c>
-      <c r="F93">
+      <c r="Q95">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A96">
+        <v>1</v>
+      </c>
+      <c r="B96">
+        <v>0</v>
+      </c>
+      <c r="C96">
+        <v>3</v>
+      </c>
+      <c r="D96">
+        <v>1</v>
+      </c>
+      <c r="E96">
+        <v>1</v>
+      </c>
+      <c r="F96">
         <v>1.76</v>
       </c>
-      <c r="G93">
+      <c r="G96">
         <v>0.12</v>
       </c>
-      <c r="H93">
+      <c r="H96">
         <v>0.22</v>
       </c>
-      <c r="I93">
+      <c r="I96">
         <v>6.8754935415698784</v>
       </c>
-      <c r="J93">
+      <c r="J96">
         <v>12.60507149287811</v>
       </c>
-      <c r="K93">
-        <v>0</v>
-      </c>
-      <c r="L93">
-        <v>0</v>
-      </c>
-      <c r="M93">
+      <c r="K96">
+        <v>0</v>
+      </c>
+      <c r="L96">
+        <v>0</v>
+      </c>
+      <c r="M96">
         <v>0.129831065</v>
       </c>
-      <c r="N93">
+      <c r="N96">
         <v>0.17618949</v>
       </c>
-      <c r="O93">
+      <c r="O96">
         <v>7.4387720741886598</v>
       </c>
-      <c r="P93">
+      <c r="P96">
         <v>10.094914171562424</v>
       </c>
-    </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A94">
-        <v>1</v>
-      </c>
-      <c r="B94">
-        <v>0</v>
-      </c>
-      <c r="C94">
-        <v>3</v>
-      </c>
-      <c r="D94">
-        <v>1</v>
-      </c>
-      <c r="E94">
-        <v>1</v>
-      </c>
-      <c r="F94">
+      <c r="Q96">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A97">
+        <v>1</v>
+      </c>
+      <c r="B97">
+        <v>0</v>
+      </c>
+      <c r="C97">
+        <v>3</v>
+      </c>
+      <c r="D97">
+        <v>1</v>
+      </c>
+      <c r="E97">
+        <v>1</v>
+      </c>
+      <c r="F97">
         <v>1.73</v>
       </c>
-      <c r="G94">
+      <c r="G97">
         <v>0.14000000000000001</v>
       </c>
-      <c r="H94">
+      <c r="H97">
         <v>0.22</v>
       </c>
-      <c r="I94">
+      <c r="I97">
         <v>8.0214091318315255</v>
       </c>
-      <c r="J94">
+      <c r="J97">
         <v>12.60507149287811</v>
       </c>
-      <c r="K94">
-        <v>0</v>
-      </c>
-      <c r="L94">
-        <v>0</v>
-      </c>
-      <c r="M94">
+      <c r="K97">
+        <v>0</v>
+      </c>
+      <c r="L97">
+        <v>0</v>
+      </c>
+      <c r="M97">
         <v>0.16908784299999999</v>
       </c>
-      <c r="N94">
+      <c r="N97">
         <v>0.14139228400000001</v>
       </c>
-      <c r="O94">
+      <c r="O97">
         <v>9.6880197708706799</v>
       </c>
-      <c r="P94">
+      <c r="P97">
         <v>8.1011811289151172</v>
       </c>
-    </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A95">
-        <v>1</v>
-      </c>
-      <c r="B95">
-        <v>0</v>
-      </c>
-      <c r="C95">
-        <v>3</v>
-      </c>
-      <c r="D95">
-        <v>1</v>
-      </c>
-      <c r="E95">
-        <v>1</v>
-      </c>
-      <c r="F95">
+      <c r="Q97">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="98" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A98">
+        <v>1</v>
+      </c>
+      <c r="B98">
+        <v>0</v>
+      </c>
+      <c r="C98">
+        <v>3</v>
+      </c>
+      <c r="D98">
+        <v>1</v>
+      </c>
+      <c r="E98">
+        <v>1</v>
+      </c>
+      <c r="F98">
         <v>1.48</v>
       </c>
-      <c r="G95">
+      <c r="G98">
         <v>0.17</v>
       </c>
-      <c r="H95">
+      <c r="H98">
         <v>0.21</v>
       </c>
-      <c r="I95">
+      <c r="I98">
         <v>9.7402825172239957</v>
       </c>
-      <c r="J95">
+      <c r="J98">
         <v>12.032113697747288</v>
       </c>
-      <c r="K95">
-        <v>0</v>
-      </c>
-      <c r="L95">
-        <v>1</v>
-      </c>
-      <c r="M95">
+      <c r="K98">
+        <v>0</v>
+      </c>
+      <c r="L98">
+        <v>1</v>
+      </c>
+      <c r="M98">
         <v>2.7919539E-2</v>
       </c>
-      <c r="N95">
+      <c r="N98">
         <v>0.13035258699999999</v>
       </c>
-      <c r="O95">
+      <c r="O98">
         <v>1.5996717506509028</v>
       </c>
-      <c r="P95">
+      <c r="P98">
         <v>7.4686530837118799</v>
       </c>
-    </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A96">
-        <v>1</v>
-      </c>
-      <c r="B96">
-        <v>0</v>
-      </c>
-      <c r="C96">
-        <v>3</v>
-      </c>
-      <c r="D96">
-        <v>1</v>
-      </c>
-      <c r="E96">
-        <v>1</v>
-      </c>
-      <c r="F96">
+      <c r="Q98">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A99">
+        <v>1</v>
+      </c>
+      <c r="B99">
+        <v>0</v>
+      </c>
+      <c r="C99">
+        <v>3</v>
+      </c>
+      <c r="D99">
+        <v>1</v>
+      </c>
+      <c r="E99">
+        <v>1</v>
+      </c>
+      <c r="F99">
         <v>1.57</v>
       </c>
-      <c r="G96">
+      <c r="G99">
         <v>0.11</v>
       </c>
-      <c r="H96">
+      <c r="H99">
         <v>0.18</v>
       </c>
-      <c r="I96">
+      <c r="I99">
         <v>6.3025357464390552</v>
       </c>
-      <c r="J96">
+      <c r="J99">
         <v>10.313240312354818</v>
       </c>
-      <c r="K96">
-        <v>0</v>
-      </c>
-      <c r="L96">
-        <v>0</v>
-      </c>
-      <c r="M96">
+      <c r="K99">
+        <v>0</v>
+      </c>
+      <c r="L99">
+        <v>0</v>
+      </c>
+      <c r="M99">
         <v>0.108239114</v>
       </c>
-      <c r="N96">
+      <c r="N99">
         <v>0.13945353199999999</v>
       </c>
-      <c r="O96">
+      <c r="O99">
         <v>6.2016444104353816</v>
       </c>
-      <c r="P96">
+      <c r="P99">
         <v>7.9900988217925688</v>
       </c>
-    </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A97">
-        <v>1</v>
-      </c>
-      <c r="B97">
-        <v>0</v>
-      </c>
-      <c r="C97">
-        <v>3</v>
-      </c>
-      <c r="D97">
-        <v>1</v>
-      </c>
-      <c r="E97">
-        <v>1</v>
-      </c>
-      <c r="F97">
+      <c r="Q99">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A100">
+        <v>1</v>
+      </c>
+      <c r="B100">
+        <v>0</v>
+      </c>
+      <c r="C100">
+        <v>3</v>
+      </c>
+      <c r="D100">
+        <v>1</v>
+      </c>
+      <c r="E100">
+        <v>1</v>
+      </c>
+      <c r="F100">
         <v>1.46</v>
       </c>
-      <c r="G97">
+      <c r="G100">
         <v>0.19</v>
       </c>
-      <c r="H97">
+      <c r="H100">
         <v>0.24</v>
       </c>
-      <c r="I97">
+      <c r="I100">
         <v>10.886198107485642</v>
       </c>
-      <c r="J97">
+      <c r="J100">
         <v>13.750987083139757</v>
       </c>
-      <c r="K97">
-        <v>0</v>
-      </c>
-      <c r="L97">
-        <v>0</v>
-      </c>
-      <c r="M97">
+      <c r="K100">
+        <v>0</v>
+      </c>
+      <c r="L100">
+        <v>0</v>
+      </c>
+      <c r="M100">
         <v>0.104937472</v>
       </c>
-      <c r="N97">
+      <c r="N100">
         <v>0.100775742</v>
       </c>
-      <c r="O97">
+      <c r="O100">
         <v>6.0124742583722499</v>
       </c>
-      <c r="P97">
+      <c r="P100">
         <v>5.7740246938992694</v>
       </c>
-    </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A98">
-        <v>1</v>
-      </c>
-      <c r="B98">
-        <v>0</v>
-      </c>
-      <c r="C98">
-        <v>3</v>
-      </c>
-      <c r="D98">
-        <v>1</v>
-      </c>
-      <c r="E98">
-        <v>1</v>
-      </c>
-      <c r="F98">
+      <c r="Q100">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="101" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A101">
+        <v>1</v>
+      </c>
+      <c r="B101">
+        <v>0</v>
+      </c>
+      <c r="C101">
+        <v>3</v>
+      </c>
+      <c r="D101">
+        <v>1</v>
+      </c>
+      <c r="E101">
+        <v>1</v>
+      </c>
+      <c r="F101">
         <v>1.45</v>
       </c>
-      <c r="G98">
+      <c r="G101">
         <v>0.21</v>
-      </c>
-      <c r="H98">
-        <v>0.19</v>
-      </c>
-      <c r="I98">
-        <v>12.032113697747288</v>
-      </c>
-      <c r="J98">
-        <v>10.886198107485642</v>
-      </c>
-      <c r="K98">
-        <v>0</v>
-      </c>
-      <c r="L98">
-        <v>0</v>
-      </c>
-      <c r="M98">
-        <v>0.14042496800000001</v>
-      </c>
-      <c r="N98">
-        <v>0.13099814300000001</v>
-      </c>
-      <c r="O98">
-        <v>8.0457580046596409</v>
-      </c>
-      <c r="P98">
-        <v>7.5056407179512297</v>
-      </c>
-    </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A99">
-        <v>1</v>
-      </c>
-      <c r="B99">
-        <v>0</v>
-      </c>
-      <c r="C99">
-        <v>3</v>
-      </c>
-      <c r="D99">
-        <v>1</v>
-      </c>
-      <c r="E99">
-        <v>1</v>
-      </c>
-      <c r="F99">
-        <v>1.83</v>
-      </c>
-      <c r="G99">
-        <v>0.18</v>
-      </c>
-      <c r="H99">
-        <v>0.2</v>
-      </c>
-      <c r="I99">
-        <v>10.313240312354818</v>
-      </c>
-      <c r="J99">
-        <v>11.459155902616466</v>
-      </c>
-      <c r="K99">
-        <v>0</v>
-      </c>
-      <c r="L99">
-        <v>1</v>
-      </c>
-      <c r="M99">
-        <v>7.0475164000000007E-2</v>
-      </c>
-      <c r="N99">
-        <v>0.10467089</v>
-      </c>
-      <c r="O99">
-        <v>4.037929457692317</v>
-      </c>
-      <c r="P99">
-        <v>5.9972002348780942</v>
-      </c>
-    </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A100">
-        <v>1</v>
-      </c>
-      <c r="B100">
-        <v>0</v>
-      </c>
-      <c r="C100">
-        <v>3</v>
-      </c>
-      <c r="D100">
-        <v>1</v>
-      </c>
-      <c r="E100">
-        <v>1</v>
-      </c>
-      <c r="F100">
-        <v>1.25</v>
-      </c>
-      <c r="G100">
-        <v>0.21</v>
-      </c>
-      <c r="H100">
-        <v>0.22</v>
-      </c>
-      <c r="I100">
-        <v>12.032113697747288</v>
-      </c>
-      <c r="J100">
-        <v>12.60507149287811</v>
-      </c>
-      <c r="K100">
-        <v>1</v>
-      </c>
-      <c r="L100">
-        <v>0</v>
-      </c>
-      <c r="M100">
-        <v>5.9086503999999998E-2</v>
-      </c>
-      <c r="N100">
-        <v>0.101203586</v>
-      </c>
-      <c r="O100">
-        <v>3.3854073053828571</v>
-      </c>
-      <c r="P100">
-        <v>5.7985383493892648</v>
-      </c>
-    </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A101">
-        <v>1</v>
-      </c>
-      <c r="B101">
-        <v>0</v>
-      </c>
-      <c r="C101">
-        <v>3</v>
-      </c>
-      <c r="D101">
-        <v>1</v>
-      </c>
-      <c r="E101">
-        <v>1</v>
-      </c>
-      <c r="F101">
-        <v>1.67</v>
-      </c>
-      <c r="G101">
-        <v>0.16</v>
       </c>
       <c r="H101">
         <v>0.19</v>
       </c>
       <c r="I101">
-        <v>9.1673247220931717</v>
+        <v>12.032113697747288</v>
       </c>
       <c r="J101">
         <v>10.886198107485642</v>
@@ -5480,279 +5783,298 @@
         <v>0</v>
       </c>
       <c r="M101">
+        <v>0.14042496800000001</v>
+      </c>
+      <c r="N101">
+        <v>0.13099814300000001</v>
+      </c>
+      <c r="O101">
+        <v>8.0457580046596409</v>
+      </c>
+      <c r="P101">
+        <v>7.5056407179512297</v>
+      </c>
+      <c r="Q101">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="102" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A102">
+        <v>1</v>
+      </c>
+      <c r="B102">
+        <v>0</v>
+      </c>
+      <c r="C102">
+        <v>3</v>
+      </c>
+      <c r="D102">
+        <v>1</v>
+      </c>
+      <c r="E102">
+        <v>1</v>
+      </c>
+      <c r="F102">
+        <v>1.83</v>
+      </c>
+      <c r="G102">
+        <v>0.18</v>
+      </c>
+      <c r="H102">
+        <v>0.2</v>
+      </c>
+      <c r="I102">
+        <v>10.313240312354818</v>
+      </c>
+      <c r="J102">
+        <v>11.459155902616466</v>
+      </c>
+      <c r="K102">
+        <v>0</v>
+      </c>
+      <c r="L102">
+        <v>1</v>
+      </c>
+      <c r="M102">
+        <v>7.0475164000000007E-2</v>
+      </c>
+      <c r="N102">
+        <v>0.10467089</v>
+      </c>
+      <c r="O102">
+        <v>4.037929457692317</v>
+      </c>
+      <c r="P102">
+        <v>5.9972002348780942</v>
+      </c>
+      <c r="Q102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A103">
+        <v>1</v>
+      </c>
+      <c r="B103">
+        <v>0</v>
+      </c>
+      <c r="C103">
+        <v>3</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
+      </c>
+      <c r="E103">
+        <v>1</v>
+      </c>
+      <c r="F103">
+        <v>1.25</v>
+      </c>
+      <c r="G103">
+        <v>0.21</v>
+      </c>
+      <c r="H103">
+        <v>0.22</v>
+      </c>
+      <c r="I103">
+        <v>12.032113697747288</v>
+      </c>
+      <c r="J103">
+        <v>12.60507149287811</v>
+      </c>
+      <c r="K103">
+        <v>1</v>
+      </c>
+      <c r="L103">
+        <v>0</v>
+      </c>
+      <c r="M103">
+        <v>5.9086503999999998E-2</v>
+      </c>
+      <c r="N103">
+        <v>0.101203586</v>
+      </c>
+      <c r="O103">
+        <v>3.3854073053828571</v>
+      </c>
+      <c r="P103">
+        <v>5.7985383493892648</v>
+      </c>
+      <c r="Q103">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A104">
+        <v>1</v>
+      </c>
+      <c r="B104">
+        <v>0</v>
+      </c>
+      <c r="C104">
+        <v>3</v>
+      </c>
+      <c r="D104">
+        <v>1</v>
+      </c>
+      <c r="E104">
+        <v>1</v>
+      </c>
+      <c r="F104">
+        <v>1.67</v>
+      </c>
+      <c r="G104">
+        <v>0.16</v>
+      </c>
+      <c r="H104">
+        <v>0.19</v>
+      </c>
+      <c r="I104">
+        <v>9.1673247220931717</v>
+      </c>
+      <c r="J104">
+        <v>10.886198107485642</v>
+      </c>
+      <c r="K104">
+        <v>0</v>
+      </c>
+      <c r="L104">
+        <v>0</v>
+      </c>
+      <c r="M104">
         <v>0.10482129900000001</v>
       </c>
-      <c r="N101">
+      <c r="N104">
         <v>0.159468361</v>
       </c>
-      <c r="O101">
+      <c r="O104">
         <v>6.0058180357788773</v>
       </c>
-      <c r="P101">
+      <c r="P104">
         <v>9.1368640511686152</v>
       </c>
-    </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A102">
-        <v>1</v>
-      </c>
-      <c r="B102">
-        <v>0</v>
-      </c>
-      <c r="C102">
-        <v>3</v>
-      </c>
-      <c r="D102">
-        <v>1</v>
-      </c>
-      <c r="E102">
-        <v>1</v>
-      </c>
-      <c r="F102">
+      <c r="Q104">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A105">
+        <v>1</v>
+      </c>
+      <c r="B105">
+        <v>0</v>
+      </c>
+      <c r="C105">
+        <v>3</v>
+      </c>
+      <c r="D105">
+        <v>1</v>
+      </c>
+      <c r="E105">
+        <v>1</v>
+      </c>
+      <c r="F105">
         <v>1.32</v>
       </c>
-      <c r="G102">
+      <c r="G105">
         <v>0.15</v>
       </c>
-      <c r="H102">
+      <c r="H105">
         <v>0.22</v>
       </c>
-      <c r="I102">
+      <c r="I105">
         <v>8.5943669269623477</v>
       </c>
-      <c r="J102">
+      <c r="J105">
         <v>12.60507149287811</v>
       </c>
-      <c r="K102">
-        <v>0</v>
-      </c>
-      <c r="L102">
-        <v>0</v>
-      </c>
-      <c r="M102">
+      <c r="K105">
+        <v>0</v>
+      </c>
+      <c r="L105">
+        <v>0</v>
+      </c>
+      <c r="M105">
         <v>9.5599726999999995E-2</v>
       </c>
-      <c r="N102">
+      <c r="N105">
         <v>0.175687179</v>
       </c>
-      <c r="O102">
+      <c r="O105">
         <v>5.4774608797028632</v>
       </c>
-      <c r="P102">
+      <c r="P105">
         <v>10.066133871259426</v>
       </c>
-    </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A103">
-        <v>1</v>
-      </c>
-      <c r="B103">
-        <v>0</v>
-      </c>
-      <c r="C103">
-        <v>3</v>
-      </c>
-      <c r="D103">
-        <v>1</v>
-      </c>
-      <c r="E103">
-        <v>1</v>
-      </c>
-      <c r="F103">
+      <c r="Q105">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A106">
+        <v>1</v>
+      </c>
+      <c r="B106">
+        <v>0</v>
+      </c>
+      <c r="C106">
+        <v>3</v>
+      </c>
+      <c r="D106">
+        <v>1</v>
+      </c>
+      <c r="E106">
+        <v>1</v>
+      </c>
+      <c r="F106">
         <v>1.6</v>
       </c>
-      <c r="G103">
+      <c r="G106">
         <v>0.18</v>
       </c>
-      <c r="H103">
+      <c r="H106">
         <v>0.18</v>
       </c>
-      <c r="I103">
+      <c r="I106">
         <v>10.313240312354818</v>
       </c>
-      <c r="J103">
+      <c r="J106">
         <v>10.313240312354818</v>
       </c>
-      <c r="K103">
-        <v>0</v>
-      </c>
-      <c r="L103">
-        <v>0</v>
-      </c>
-      <c r="M103">
+      <c r="K106">
+        <v>0</v>
+      </c>
+      <c r="L106">
+        <v>0</v>
+      </c>
+      <c r="M106">
         <v>0.12110438699999999</v>
       </c>
-      <c r="N103">
+      <c r="N106">
         <v>3.6538968999999998E-2</v>
       </c>
-      <c r="O103">
+      <c r="O106">
         <v>6.9387702556189934</v>
       </c>
-      <c r="P103">
+      <c r="P106">
         <v>2.0935287114593497</v>
       </c>
-    </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A104">
-        <v>1</v>
-      </c>
-      <c r="B104">
-        <v>1</v>
-      </c>
-      <c r="C104">
-        <v>3</v>
-      </c>
-      <c r="D104">
-        <v>1</v>
-      </c>
-      <c r="E104">
-        <v>1</v>
-      </c>
-      <c r="F104">
-        <v>2.23</v>
-      </c>
-      <c r="G104">
-        <v>0.21</v>
-      </c>
-      <c r="H104">
-        <v>0.21</v>
-      </c>
-      <c r="I104">
-        <v>12.032113697747288</v>
-      </c>
-      <c r="J104">
-        <v>12.032113697747288</v>
-      </c>
-      <c r="K104">
-        <v>0</v>
-      </c>
-      <c r="L104">
-        <v>1</v>
-      </c>
-      <c r="M104">
-        <v>0.160054637</v>
-      </c>
-      <c r="N104">
-        <v>0.162121971</v>
-      </c>
-      <c r="O104">
-        <v>9.1704551915984283</v>
-      </c>
-      <c r="P104">
-        <v>9.2889047046423272</v>
-      </c>
-    </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A105">
-        <v>1</v>
-      </c>
-      <c r="B105">
-        <v>1</v>
-      </c>
-      <c r="C105">
-        <v>3</v>
-      </c>
-      <c r="D105">
-        <v>1</v>
-      </c>
-      <c r="E105">
-        <v>1</v>
-      </c>
-      <c r="F105">
-        <v>1.83</v>
-      </c>
-      <c r="G105">
-        <v>0.11</v>
-      </c>
-      <c r="H105">
-        <v>0.18</v>
-      </c>
-      <c r="I105">
-        <v>6.3025357464390552</v>
-      </c>
-      <c r="J105">
-        <v>10.313240312354818</v>
-      </c>
-      <c r="K105">
-        <v>0</v>
-      </c>
-      <c r="L105">
-        <v>1</v>
-      </c>
-      <c r="M105">
-        <v>0.19846751800000001</v>
-      </c>
-      <c r="N105">
-        <v>0.18295019200000001</v>
-      </c>
-      <c r="O105">
-        <v>11.371351151836697</v>
-      </c>
-      <c r="P105">
-        <v>10.482273862708078</v>
-      </c>
-    </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A106">
-        <v>1</v>
-      </c>
-      <c r="B106">
-        <v>1</v>
-      </c>
-      <c r="C106">
-        <v>3</v>
-      </c>
-      <c r="D106">
-        <v>1</v>
-      </c>
-      <c r="E106">
-        <v>1</v>
-      </c>
-      <c r="F106">
-        <v>1.58</v>
-      </c>
-      <c r="G106">
-        <v>0.17</v>
-      </c>
-      <c r="H106">
-        <v>0.22</v>
-      </c>
-      <c r="I106">
-        <v>9.7402825172239957</v>
-      </c>
-      <c r="J106">
-        <v>12.60507149287811</v>
-      </c>
-      <c r="K106">
-        <v>0</v>
-      </c>
-      <c r="L106">
-        <v>0</v>
-      </c>
-      <c r="M106">
-        <v>0.185135622</v>
-      </c>
-      <c r="N106">
-        <v>0.14476037899999999</v>
-      </c>
-      <c r="O106">
-        <v>10.607489778129352</v>
-      </c>
-      <c r="P106">
-        <v>8.2941587574142321</v>
-      </c>
-    </row>
+      <c r="Q106">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:17" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="108" spans="1:17" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="109" spans="1:17" hidden="1" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <autoFilter ref="B1:B109" xr:uid="{C9F0F03B-9386-4C50-90B6-016F7CF3CBF2}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" copies="0" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A87BD8E3-760C-4CCC-8501-E9647EAEFB82}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>